<commit_message>
Log nonlinear system build + live confirmation to the FRF study write-up
Part G: build/validation of the amplitude-dependent (Duffing-softening +
quadratic-damping) mode-1 nonlinear system, the RK4 accuracy bug caught
and fixed along the way, the four separate hardware-dispatch wiring gaps
found and fixed, and the live -6/0/+12dB confirmation that optimal_
diagonal_control's FRF-drift tracking holds response error flat across
an 8x drive-amplitude swing -- including the corrected post-hoc modal-
amplitude analysis (an initial units-error false alarm, then the
corrected calculation showing the system is comfortably stable) and
confirmation that the softened mode-1 peak is visible in the measured
FRF on channels 7/8.

Profile file reflects the current test configuration used for that
live confirmation (hardware type 7 / nonlinear system, standard
optimal_diagonal_control).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sixdrive12resp/results/sdynpy_frame6x12_profile.xlsx
+++ b/examples/sixdrive12resp/results/sdynpy_frame6x12_profile.xlsx
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C1" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/Users/nhunterjr/Documents/Code/python/rattlesnake-vibration-controller/examples/sixdrive12resp/results/sdynpy_frame6x12_system.npz</t>
+          <t>/Users/nhunterjr/Documents/Code/python/rattlesnake-vibration-controller/examples/sixdrive12resp/results/sdynpy_frame6x12_system_nonlinear.npz</t>
         </is>
       </c>
     </row>

</xml_diff>